<commit_message>
remind logic/code to apply java threads
</commit_message>
<xml_diff>
--- a/src/main/resources/excel/students.xlsx
+++ b/src/main/resources/excel/students.xlsx
@@ -125,7 +125,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="n" s="2">
-        <v>23.0</v>
+        <v>21.0</v>
       </c>
       <c r="D2" t="s" s="2">
         <v>5</v>
@@ -139,7 +139,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="n" s="2">
-        <v>25.0</v>
+        <v>21.0</v>
       </c>
       <c r="D3" t="s" s="2">
         <v>7</v>
@@ -153,7 +153,7 @@
         <v>8</v>
       </c>
       <c r="C4" t="n" s="2">
-        <v>23.0</v>
+        <v>19.0</v>
       </c>
       <c r="D4" t="s" s="2">
         <v>5</v>

</xml_diff>